<commit_message>
feat: presupuesto personal junio 2026 - Excel
</commit_message>
<xml_diff>
--- a/EXCEL/Reporte-Ventas-TiendaDB.xlsx
+++ b/EXCEL/Reporte-Ventas-TiendaDB.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{89DC2EF8-6C9A-442A-AEF9-25CB1F4797E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-192" yWindow="348" windowWidth="11268" windowHeight="9840" firstSheet="2" activeTab="3" xr2:uid="{7A69F9BD-A0FC-4DDD-AC3B-D154E30BA4F1}"/>
+    <workbookView xWindow="-48" yWindow="2964" windowWidth="11268" windowHeight="9840" firstSheet="2" activeTab="3" xr2:uid="{7A69F9BD-A0FC-4DDD-AC3B-D154E30BA4F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Ventas-Producto" sheetId="1" r:id="rId1"/>
@@ -227,21 +227,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1300,6 +1299,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-D59F-4FA6-8AAF-94CA43F6F937}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -1317,6 +1321,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-D59F-4FA6-8AAF-94CA43F6F937}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -1468,6 +1477,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-D59F-4FA6-8AAF-94CA43F6F937}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -1481,6 +1495,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-D59F-4FA6-8AAF-94CA43F6F937}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -1494,6 +1513,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000D-D59F-4FA6-8AAF-94CA43F6F937}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -1507,6 +1531,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000F-D59F-4FA6-8AAF-94CA43F6F937}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -6989,7 +7018,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2309091-4879-4057-95CE-848B0AF45375}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -6998,79 +7027,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="7">
         <v>1</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2" s="7">
         <v>45.99</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="7">
         <v>1</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="7">
         <v>39.99</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
         <v>2</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <v>3</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <v>1</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="7">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="7">
         <v>2</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="7">
         <v>17</v>
       </c>
     </row>
@@ -7078,31 +7107,6 @@
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:C7" xr:uid="{E2309091-4879-4057-95CE-848B0AF45375}">
@@ -7127,68 +7131,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>1</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="6">
         <v>39.99</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>1</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="6">
         <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>1</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>1</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>62.99</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>1</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>37</v>
       </c>
     </row>
@@ -7215,57 +7219,57 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="5">
         <v>2</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <v>98.99</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="5">
         <v>1</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="5">
         <v>39.99</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="5">
         <v>1</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="5">
         <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="5">
         <v>1</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <v>25</v>
       </c>
     </row>
@@ -7285,14 +7289,14 @@
   <dimension ref="E1:K3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="4" width="8.88671875" style="9"/>
-    <col min="5" max="6" width="8.88671875" style="9" customWidth="1"/>
-    <col min="7" max="9" width="8.88671875" style="9"/>
-    <col min="10" max="10" width="15.88671875" style="9" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="9"/>
+    <col min="1" max="4" width="8.88671875" style="8"/>
+    <col min="5" max="6" width="8.88671875" style="8" customWidth="1"/>
+    <col min="7" max="9" width="8.88671875" style="8"/>
+    <col min="10" max="10" width="15.88671875" style="8" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="5:11" s="9" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="5:11" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G1" s="10" t="s">
         <v>22</v>
       </c>
@@ -7301,21 +7305,21 @@
       <c r="J1" s="10"/>
       <c r="K1" s="10"/>
     </row>
-    <row r="2" spans="5:11" s="9" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="5:11" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
       <c r="I2" s="10"/>
       <c r="J2" s="10"/>
       <c r="K2" s="10"/>
     </row>
-    <row r="3" spans="5:11" s="9" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
+    <row r="3" spans="5:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>